<commit_message>
Añado la eliminación de archivos al iniciar una nueva sesión
</commit_message>
<xml_diff>
--- a/registros_citas.xlsx
+++ b/registros_citas.xlsx
@@ -50,40 +50,40 @@
     <t>Enlace (si es virtual)</t>
   </si>
   <si>
-    <t>Danna</t>
-  </si>
-  <si>
-    <t>12345678A</t>
-  </si>
-  <si>
-    <t>600123123</t>
-  </si>
-  <si>
-    <t>Alejandro</t>
-  </si>
-  <si>
-    <t>99887766B</t>
-  </si>
-  <si>
-    <t>General</t>
+    <t>Maria Paula</t>
+  </si>
+  <si>
+    <t>987654</t>
+  </si>
+  <si>
+    <t>564789</t>
+  </si>
+  <si>
+    <t>Juan Camilo</t>
+  </si>
+  <si>
+    <t>123456</t>
+  </si>
+  <si>
+    <t>Ginecología</t>
   </si>
   <si>
     <t>2025</t>
   </si>
   <si>
-    <t>05</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>16:00</t>
-  </si>
-  <si>
-    <t>Presencial</t>
-  </si>
-  <si>
-    <t>-</t>
+    <t>04</t>
+  </si>
+  <si>
+    <t>07</t>
+  </si>
+  <si>
+    <t>05:00</t>
+  </si>
+  <si>
+    <t>Virtual</t>
+  </si>
+  <si>
+    <t>https://www.uaoepsmeet.com/123456</t>
   </si>
 </sst>
 </file>

</xml_diff>